<commit_message>
- grounded framing statistics
</commit_message>
<xml_diff>
--- a/DFN_lex_stats.xlsx
+++ b/DFN_lex_stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/piek/Desktop/DFN-final/OpenDutchFrameNetLexicon/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAD04C8F-CCB3-624A-952A-E605C50346A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3472457F-4E44-3D4F-989D-1360997BB729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3800" yWindow="2600" windowWidth="28240" windowHeight="17240" xr2:uid="{DA26D9AA-C628-7245-AC36-110158425BD4}"/>
+    <workbookView xWindow="2380" yWindow="1760" windowWidth="28240" windowHeight="17240" activeTab="3" xr2:uid="{DA26D9AA-C628-7245-AC36-110158425BD4}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="510">
   <si>
     <t>nl_reference_lexicon.json</t>
   </si>
@@ -1413,13 +1413,169 @@
   </si>
   <si>
     <t>Lexicon</t>
+  </si>
+  <si>
+    <t>Frames per entry</t>
+  </si>
+  <si>
+    <t>Annotation per entry</t>
+  </si>
+  <si>
+    <t>Frame coverage</t>
+  </si>
+  <si>
+    <t>Manual annotations</t>
+  </si>
+  <si>
+    <t>Lexical baseline</t>
+  </si>
+  <si>
+    <t>Dutch Framenet v1.0</t>
+  </si>
+  <si>
+    <t>Counts</t>
+  </si>
+  <si>
+    <t>Data2Text annotations</t>
+  </si>
+  <si>
+    <t>RBN-Wordnet mappings</t>
+  </si>
+  <si>
+    <t>Sonar annotations</t>
+  </si>
+  <si>
+    <t>fn17-statement@speaker:</t>
+  </si>
+  <si>
+    <t>fn17-responsibility@agent:</t>
+  </si>
+  <si>
+    <t>fn17-affirm\_or\_deny@speaker:</t>
+  </si>
+  <si>
+    <t>fn17-criminal\_investigation@suspect:</t>
+  </si>
+  <si>
+    <t>fn17-supply@supplier:</t>
+  </si>
+  <si>
+    <t>fn17-exchange@exchanger\_1:</t>
+  </si>
+  <si>
+    <t>Q159 (Russia)</t>
+  </si>
+  <si>
+    <t>NL</t>
+  </si>
+  <si>
+    <t>EN</t>
+  </si>
+  <si>
+    <t>NL&amp;EN</t>
+  </si>
+  <si>
+    <t>fn17-offenses@perpetrator</t>
+  </si>
+  <si>
+    <t>fn17-suspicion@suspect</t>
+  </si>
+  <si>
+    <t>fn17-hit_target@agent</t>
+  </si>
+  <si>
+    <t>fn17-attack@assailant</t>
+  </si>
+  <si>
+    <t>fn17-killing@killer</t>
+  </si>
+  <si>
+    <t>fn17-terrorism@terrorist</t>
+  </si>
+  <si>
+    <t>fn17-suspicion</t>
+  </si>
+  <si>
+    <t>fn17-trial@defendant</t>
+  </si>
+  <si>
+    <t>fn17-statement@speaker</t>
+  </si>
+  <si>
+    <t>fn17-committing_crime@perpetrator</t>
+  </si>
+  <si>
+    <t>fn17-use_firearm@agent</t>
+  </si>
+  <si>
+    <t>fn17-arrest@suspect</t>
+  </si>
+  <si>
+    <t>fn17-detaining@suspect</t>
+  </si>
+  <si>
+    <t>fn17-bearing_arms</t>
+  </si>
+  <si>
+    <t>}</t>
+  </si>
+  <si>
+    <t>fn17-chaos@entity</t>
+  </si>
+  <si>
+    <t>fn17-chaos@state</t>
+  </si>
+  <si>
+    <t>fn17-chaos</t>
+  </si>
+  <si>
+    <t>fn17-people</t>
+  </si>
+  <si>
+    <t>fn17-robbery@perpetrator</t>
+  </si>
+  <si>
+    <t>fn17-emotion_directed@experiencer</t>
+  </si>
+  <si>
+    <t>fn17-verdict@defendant</t>
+  </si>
+  <si>
+    <t>fn17-setting_fire@kindler</t>
+  </si>
+  <si>
+    <t>fn17-hostile_encounter@side_2</t>
+  </si>
+  <si>
+    <t>rioter</t>
+  </si>
+  <si>
+    <t>fn17-protest@protester</t>
+  </si>
+  <si>
+    <t>fn17-causation@actor</t>
+  </si>
+  <si>
+    <t>fn17-cause_harm@agent</t>
+  </si>
+  <si>
+    <t>fn17-damaging@agent</t>
+  </si>
+  <si>
+    <t>fn17-destroying@destroyer</t>
+  </si>
+  <si>
+    <t>fn17-evading@evader</t>
+  </si>
+  <si>
+    <t>fn17-resolve_problem@problem</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1433,6 +1589,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFBCBEC4"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1491,21 +1653,23 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1841,7 +2005,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60F15FF6-B794-844A-AEFB-D94A9258D4AF}">
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="41.83203125" bestFit="1" customWidth="1"/>
@@ -2391,8 +2555,139 @@
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>463</v>
+      </c>
+      <c r="B20" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>312</v>
+      </c>
+      <c r="B21" s="11">
+        <f>SUM(B4)</f>
+        <v>6964</v>
+      </c>
+    </row>
     <row r="22" spans="1:5">
-      <c r="A22" s="9"/>
+      <c r="A22" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="B22" s="11">
+        <f>SUM(C4)</f>
+        <v>2883</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>316</v>
+      </c>
+      <c r="B23" s="11">
+        <f>SUM(D4)</f>
+        <v>218</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>314</v>
+      </c>
+      <c r="B24" s="11">
+        <f>SUM(E4)</f>
+        <v>2621</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>315</v>
+      </c>
+      <c r="B25" s="11">
+        <f>SUM(F4)</f>
+        <v>530</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>458</v>
+      </c>
+      <c r="B26" s="12">
+        <f>SUM(G4)</f>
+        <v>3.0134141064474198</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>459</v>
+      </c>
+      <c r="B27" s="12">
+        <f>SUM(H4)</f>
+        <v>12.405884898312401</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>328</v>
+      </c>
+      <c r="B28" s="11">
+        <f>SUM(I4)</f>
+        <v>28670</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" t="s">
+        <v>460</v>
+      </c>
+      <c r="B29" s="11">
+        <f>SUM(J4)</f>
+        <v>2311</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" t="s">
+        <v>461</v>
+      </c>
+      <c r="B30" s="11">
+        <f>SUM(K4)</f>
+        <v>27841</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" t="s">
+        <v>462</v>
+      </c>
+      <c r="B31" s="11">
+        <f>SUM(L4)</f>
+        <v>829</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" t="s">
+        <v>465</v>
+      </c>
+      <c r="B32" s="11">
+        <f>SUM(M4)</f>
+        <v>22435</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>466</v>
+      </c>
+      <c r="B33" s="11">
+        <f>SUM(N4)</f>
+        <v>954</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>467</v>
+      </c>
+      <c r="B34" s="11">
+        <f>SUM(O4)</f>
+        <v>5281</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2401,14 +2696,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58832A8D-FB52-9244-8B18-6ED143CEC1A5}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:E138"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="41.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.5" customWidth="1"/>
+    <col min="3" max="3" width="40" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>176</v>
       </c>
@@ -2419,7 +2716,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>177</v>
       </c>
@@ -2430,7 +2727,7 @@
         <v>9588</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>176</v>
       </c>
@@ -2441,7 +2738,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>177</v>
       </c>
@@ -2452,7 +2749,7 @@
         <v>37536</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -2460,7 +2757,603 @@
         <v>171</v>
       </c>
     </row>
+    <row r="8" spans="1:5">
+      <c r="B8" t="s">
+        <v>474</v>
+      </c>
+      <c r="C8" t="s">
+        <v>477</v>
+      </c>
+      <c r="D8" t="s">
+        <v>475</v>
+      </c>
+      <c r="E8" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="B9" t="s">
+        <v>468</v>
+      </c>
+      <c r="C9">
+        <v>55</v>
+      </c>
+      <c r="D9">
+        <v>13</v>
+      </c>
+      <c r="E9">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="B10" t="s">
+        <v>469</v>
+      </c>
+      <c r="C10">
+        <v>48</v>
+      </c>
+      <c r="D10">
+        <v>36</v>
+      </c>
+      <c r="E10">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="B11" t="s">
+        <v>470</v>
+      </c>
+      <c r="C11">
+        <v>47</v>
+      </c>
+      <c r="D11">
+        <v>12</v>
+      </c>
+      <c r="E11">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="B12" t="s">
+        <v>471</v>
+      </c>
+      <c r="C12">
+        <v>37</v>
+      </c>
+      <c r="D12">
+        <v>23</v>
+      </c>
+      <c r="E12">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="B13" t="s">
+        <v>472</v>
+      </c>
+      <c r="C13">
+        <v>34</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="B14" t="s">
+        <v>473</v>
+      </c>
+      <c r="C14">
+        <v>22</v>
+      </c>
+      <c r="D14">
+        <v>5</v>
+      </c>
+      <c r="E14">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="B15" t="s">
+        <v>287</v>
+      </c>
+      <c r="C15" t="s">
+        <v>477</v>
+      </c>
+      <c r="D15" t="s">
+        <v>475</v>
+      </c>
+      <c r="E15" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="B16" t="s">
+        <v>478</v>
+      </c>
+      <c r="C16">
+        <v>39</v>
+      </c>
+      <c r="D16">
+        <v>19</v>
+      </c>
+      <c r="E16">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5">
+      <c r="B17" t="s">
+        <v>479</v>
+      </c>
+      <c r="C17">
+        <v>33</v>
+      </c>
+      <c r="D17">
+        <v>11</v>
+      </c>
+      <c r="E17">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5">
+      <c r="B18" t="s">
+        <v>480</v>
+      </c>
+      <c r="C18">
+        <v>29</v>
+      </c>
+      <c r="D18">
+        <v>17</v>
+      </c>
+      <c r="E18">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5">
+      <c r="B19" t="s">
+        <v>481</v>
+      </c>
+      <c r="C19">
+        <v>25</v>
+      </c>
+      <c r="D19">
+        <v>13</v>
+      </c>
+      <c r="E19">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" t="s">
+        <v>482</v>
+      </c>
+      <c r="C20">
+        <v>22</v>
+      </c>
+      <c r="D20">
+        <v>8</v>
+      </c>
+      <c r="E20">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5">
+      <c r="B21" t="s">
+        <v>483</v>
+      </c>
+      <c r="C21">
+        <v>22</v>
+      </c>
+      <c r="D21">
+        <v>15</v>
+      </c>
+      <c r="E21">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5">
+      <c r="B22" t="s">
+        <v>484</v>
+      </c>
+      <c r="C22">
+        <v>21</v>
+      </c>
+      <c r="D22">
+        <v>7</v>
+      </c>
+      <c r="E22">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5">
+      <c r="B23" t="s">
+        <v>485</v>
+      </c>
+      <c r="C23">
+        <v>19</v>
+      </c>
+      <c r="D23">
+        <v>14</v>
+      </c>
+      <c r="E23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5">
+      <c r="B24" t="s">
+        <v>486</v>
+      </c>
+      <c r="C24">
+        <v>11</v>
+      </c>
+      <c r="D24">
+        <v>9</v>
+      </c>
+      <c r="E24">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25" t="s">
+        <v>487</v>
+      </c>
+      <c r="C25">
+        <v>12</v>
+      </c>
+      <c r="D25">
+        <v>8</v>
+      </c>
+      <c r="E25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5">
+      <c r="B26" t="s">
+        <v>488</v>
+      </c>
+      <c r="C26">
+        <v>15</v>
+      </c>
+      <c r="D26">
+        <v>3</v>
+      </c>
+      <c r="E26">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5">
+      <c r="B27" t="s">
+        <v>489</v>
+      </c>
+      <c r="C27">
+        <v>13</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5">
+      <c r="B28" t="s">
+        <v>490</v>
+      </c>
+      <c r="C28">
+        <v>15</v>
+      </c>
+      <c r="D28">
+        <v>4</v>
+      </c>
+      <c r="E28">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5">
+      <c r="B29" t="s">
+        <v>491</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <v>0</v>
+      </c>
+      <c r="E29">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5">
+      <c r="B32" t="s">
+        <v>502</v>
+      </c>
+      <c r="C32" t="s">
+        <v>477</v>
+      </c>
+      <c r="D32" t="s">
+        <v>475</v>
+      </c>
+      <c r="E32" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5">
+      <c r="B33" t="s">
+        <v>493</v>
+      </c>
+      <c r="C33">
+        <v>19</v>
+      </c>
+      <c r="D33">
+        <v>11</v>
+      </c>
+      <c r="E33">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5">
+      <c r="B34" t="s">
+        <v>494</v>
+      </c>
+      <c r="C34">
+        <v>5</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5">
+      <c r="B35" t="s">
+        <v>495</v>
+      </c>
+      <c r="C35">
+        <v>5</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5">
+      <c r="B36" t="s">
+        <v>487</v>
+      </c>
+      <c r="C36">
+        <v>4</v>
+      </c>
+      <c r="D36">
+        <v>3</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5">
+      <c r="B37" t="s">
+        <v>496</v>
+      </c>
+      <c r="C37">
+        <v>4</v>
+      </c>
+      <c r="D37">
+        <v>3</v>
+      </c>
+      <c r="E37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5">
+      <c r="B38" s="9" t="s">
+        <v>497</v>
+      </c>
+      <c r="C38">
+        <v>2</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5">
+      <c r="B39" t="s">
+        <v>498</v>
+      </c>
+      <c r="C39">
+        <v>2</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5">
+      <c r="B40" t="s">
+        <v>499</v>
+      </c>
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5">
+      <c r="B41" t="s">
+        <v>500</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5">
+      <c r="B42" t="s">
+        <v>501</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5">
+      <c r="B43" t="s">
+        <v>503</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>9</v>
+      </c>
+      <c r="E43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5">
+      <c r="B44" t="s">
+        <v>481</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>8</v>
+      </c>
+      <c r="E44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5">
+      <c r="B45" t="s">
+        <v>504</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>6</v>
+      </c>
+      <c r="E45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5">
+      <c r="B46" t="s">
+        <v>489</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>5</v>
+      </c>
+      <c r="E46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5">
+      <c r="B47" t="s">
+        <v>505</v>
+      </c>
+      <c r="C47">
+        <v>0</v>
+      </c>
+      <c r="D47">
+        <v>5</v>
+      </c>
+      <c r="E47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5">
+      <c r="B48" t="s">
+        <v>506</v>
+      </c>
+      <c r="C48">
+        <v>0</v>
+      </c>
+      <c r="D48">
+        <v>4</v>
+      </c>
+      <c r="E48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5">
+      <c r="B49" t="s">
+        <v>507</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+      <c r="D49">
+        <v>4</v>
+      </c>
+      <c r="E49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5">
+      <c r="B50" t="s">
+        <v>508</v>
+      </c>
+      <c r="C50">
+        <v>2</v>
+      </c>
+      <c r="D50">
+        <v>0</v>
+      </c>
+      <c r="E50">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5">
+      <c r="B51" t="s">
+        <v>509</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51">
+        <v>0</v>
+      </c>
+      <c r="E51">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="138" spans="2:2">
+      <c r="B138" s="13" t="s">
+        <v>492</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B38" r:id="rId1" xr:uid="{5FCEBA52-C7DD-844A-A202-CC847A0F39E4}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>